<commit_message>
colorize ^ True False binary input
</commit_message>
<xml_diff>
--- a/MBN Preprocessing/VIF_results.xlsx
+++ b/MBN Preprocessing/VIF_results.xlsx
@@ -447,7 +447,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>68.96718512709668</v>
+        <v>169.3481497267666</v>
       </c>
     </row>
     <row r="3">
@@ -457,7 +457,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>68.81818375725591</v>
+        <v>169.2334036316672</v>
       </c>
     </row>
     <row r="4">
@@ -467,7 +467,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1.35421223931369</v>
+        <v>1.328366572877282</v>
       </c>
     </row>
     <row r="5">
@@ -477,7 +477,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1.317693429380591</v>
+        <v>1.3098340033045</v>
       </c>
     </row>
     <row r="6">
@@ -487,7 +487,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1.106134465458524</v>
+        <v>1.103697571826028</v>
       </c>
     </row>
     <row r="7">
@@ -497,7 +497,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1.051847502231949</v>
+        <v>1.036836961126542</v>
       </c>
     </row>
     <row r="8">
@@ -507,7 +507,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1.017166044238083</v>
+        <v>1.017752368739366</v>
       </c>
     </row>
   </sheetData>

</xml_diff>